<commit_message>
SDS library: add Slide Resin Remover, current US SDSs for Coleman and Bissell, archive duplicates, PPE icons
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L8GjKHSsuRpbp1LK9h1qLQ
</commit_message>
<xml_diff>
--- a/sds/SDS-Register.xlsx
+++ b/sds/SDS-Register.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Register'!$A$1:$U$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Register'!$A$1:$U$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -96,7 +95,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -122,10 +121,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -664,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U99"/>
+  <dimension ref="A1:U100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -841,10 +843,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J2" s="9" t="n">
+      <c r="J2" s="11" t="n">
         <v>45685</v>
       </c>
-      <c r="K2" s="9" t="n">
+      <c r="K2" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L2" s="7" t="inlineStr">
@@ -942,10 +944,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands</t>
         </is>
       </c>
-      <c r="J3" s="9" t="n">
+      <c r="J3" s="11" t="n">
         <v>42153</v>
       </c>
-      <c r="K3" s="9" t="n">
+      <c r="K3" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L3" s="7" t="inlineStr">
@@ -1051,10 +1053,10 @@
       </c>
       <c r="H4" s="8" t="inlineStr"/>
       <c r="I4" s="8" t="inlineStr"/>
-      <c r="J4" s="9" t="n">
+      <c r="J4" s="11" t="n">
         <v>43349</v>
       </c>
-      <c r="K4" s="9" t="n">
+      <c r="K4" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
@@ -1167,10 +1169,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J5" s="9" t="n">
+      <c r="J5" s="11" t="n">
         <v>46316</v>
       </c>
-      <c r="K5" s="9" t="n">
+      <c r="K5" s="11" t="n">
         <v>46316</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -1260,10 +1262,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J6" s="9" t="n">
+      <c r="J6" s="11" t="n">
         <v>46316</v>
       </c>
-      <c r="K6" s="9" t="n">
+      <c r="K6" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -1353,10 +1355,10 @@
           <t>Wear eye protection; Wear protective gloves</t>
         </is>
       </c>
-      <c r="J7" s="9" t="n">
+      <c r="J7" s="11" t="n">
         <v>45604</v>
       </c>
-      <c r="K7" s="9" t="n">
+      <c r="K7" s="11" t="n">
         <v>46315</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -1416,10 +1418,10 @@
       <c r="G8" s="7" t="inlineStr"/>
       <c r="H8" s="8" t="inlineStr"/>
       <c r="I8" s="8" t="inlineStr"/>
-      <c r="J8" s="9" t="n">
+      <c r="J8" s="11" t="n">
         <v>39855</v>
       </c>
-      <c r="K8" s="9" t="n">
+      <c r="K8" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -1511,10 +1513,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J9" s="9" t="n">
+      <c r="J9" s="11" t="n">
         <v>44131</v>
       </c>
-      <c r="K9" s="9" t="n">
+      <c r="K9" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
@@ -1621,8 +1623,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n">
+      <c r="J10" s="11" t="n"/>
+      <c r="K10" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -1700,12 +1702,12 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Coleman Fuel</t>
+          <t>Coleman Camp Fuel</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>Coleman UK plc</t>
+          <t>The Coleman Company, Inc.</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -1719,15 +1721,29 @@
           <t>Danger</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="8" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>GHS02, GHS07, GHS08</t>
+        </is>
+      </c>
+      <c r="H11" s="8" t="inlineStr">
+        <is>
+          <t>H225 Highly flammable liquid and vapor
+H304 May be fatal if swallowed and enters airways
+H336 May cause drowsiness or dizziness
+H361 Suspected of damaging fertility or the unborn child
+H411 Toxic to aquatic life with long lasting effects</t>
+        </is>
+      </c>
       <c r="I11" s="8" t="inlineStr">
         <is>
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n">
+      <c r="J11" s="11" t="n">
+        <v>44658</v>
+      </c>
+      <c r="K11" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L11" s="7" t="inlineStr">
@@ -1735,48 +1751,35 @@
           <t>3370910.pdf</t>
         </is>
       </c>
-      <c r="M11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr">
+        <is>
+          <t>(800) 424-9300</t>
+        </is>
+      </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
           <t>Active</t>
         </is>
       </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>UK sheet with old EU risk phrases, not a US GHS SDS. Get the current US SDS from Coleman.</t>
-        </is>
-      </c>
+      <c r="O11" s="8" t="n"/>
       <c r="P11" s="8" t="inlineStr">
         <is>
-          <t>Skin: May cause irritation to skin. Wash off immediately with plenty of soap and water. Remove contaminated clothing. Seek medical attention if irritation or symptoms persist.
-Eyes: May cause irritation to eyes. Rinse immediately with plenty of water for 15 minutes holding the eyelids open. Seek medical attention if irritation or symptoms persist.
-Inhalation: Inhalation may cause coughing, tightness of the chest and irritation of the respiratory system. Move the exposed person to fresh air. Seek medical attention.
-Swallowed: Ingestion may cause nausea and vomiting. Seek medical attention if irritation or symptoms persist.
-General: In case of accident or if you feel unwell, seek medical advice immediately (show the label where possible).</t>
-        </is>
-      </c>
-      <c r="Q11" s="8" t="inlineStr">
-        <is>
-          <t>Extinguishing media: Carbon dioxide (CO2) Alcohol resistant foam.
-Fire hazard: Highly flammable. Vapour may travel considerable distance to source of ignition and flash back.
-Special protective actions for fire-fighters: Wear suitable respiratory equipment when necessary.</t>
-        </is>
-      </c>
-      <c r="R11" s="8" t="inlineStr">
-        <is>
-          <t>Personal precautions, protective equipment and emergency procedures: Ensure adequate ventilation of the working area. Evacuate personnel to a safe area. Eliminate all sources of ignition. Wear suitable protective equipment.
-Environmental precautions: Do not allow product to enter drains. Prevent further spillage if safe. Inform repective authorities in case of seepage into water course or sewage system.
-Methods and material for containment and cleaning up: Absorb with inert, absorbent material. Transfer to suitable, labelled containers for disposal. Clean spillage area thoroughly with plenty of water. Endsure adequate ventilation.</t>
-        </is>
-      </c>
-      <c r="S11" s="8" t="inlineStr">
-        <is>
-          <t>Precautions for safe handling: Avoid contact with eyes and skin. Ensure adequate ventilation of the working area. Use explosion proof equipment. Keep away from sources of ignition - No smoking.
-Conditions for safe storage, including any incompatibilities: Keep in a cool, dry, well ventilated area. Keep containers tightly closed. Store in correctly labelled containers.</t>
-        </is>
-      </c>
-      <c r="T11" s="8" t="inlineStr"/>
-      <c r="U11" s="8" t="inlineStr"/>
+          <t>General: If exposed or concerned, get medical attention. Show this SDS to the doctor.
+Inhalation: Remove to fresh air and keep at rest. Get medical attention. If breathing is difficult, supply oxygen.
+Skin: Remove affected clothing and wash exposed skin with water for at least 15 minutes. Get medical attention if irritation persists.
+Eyes: Flush with plenty of water for at least 15 minutes. Remove contact lenses if easy. Get medical attention if irritation persists.
+Swallowed: Rinse mouth. Do NOT induce vomiting. Get medical attention immediately (aspiration hazard).</t>
+        </is>
+      </c>
+      <c r="Q11" s="8" t="n"/>
+      <c r="R11" s="8" t="n"/>
+      <c r="S11" s="8" t="n"/>
+      <c r="T11" s="8" t="n"/>
+      <c r="U11" s="8" t="inlineStr">
+        <is>
+          <t>Replaced 10/22/2026: the old UK sheet was swapped for the current US GHS SDS (The Coleman Company, rev. 04/07/2022).</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="45" customHeight="1">
       <c r="A12" s="7" t="n">
@@ -1806,10 +1809,10 @@
       <c r="G12" s="7" t="inlineStr"/>
       <c r="H12" s="8" t="inlineStr"/>
       <c r="I12" s="8" t="inlineStr"/>
-      <c r="J12" s="9" t="n">
+      <c r="J12" s="11" t="n">
         <v>42167</v>
       </c>
-      <c r="K12" s="9" t="n">
+      <c r="K12" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -1904,10 +1907,10 @@
       </c>
       <c r="H13" s="8" t="inlineStr"/>
       <c r="I13" s="8" t="inlineStr"/>
-      <c r="J13" s="9" t="n">
+      <c r="J13" s="11" t="n">
         <v>45247</v>
       </c>
-      <c r="K13" s="9" t="n">
+      <c r="K13" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -2006,10 +2009,10 @@
       </c>
       <c r="H14" s="8" t="inlineStr"/>
       <c r="I14" s="8" t="inlineStr"/>
-      <c r="J14" s="9" t="n">
+      <c r="J14" s="11" t="n">
         <v>42129</v>
       </c>
-      <c r="K14" s="9" t="n">
+      <c r="K14" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
@@ -2099,10 +2102,10 @@
       </c>
       <c r="H15" s="8" t="inlineStr"/>
       <c r="I15" s="8" t="inlineStr"/>
-      <c r="J15" s="9" t="n">
+      <c r="J15" s="11" t="n">
         <v>42114</v>
       </c>
-      <c r="K15" s="9" t="n">
+      <c r="K15" s="11" t="n">
         <v>46266</v>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -2200,8 +2203,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J16" s="9" t="n"/>
-      <c r="K16" s="9" t="n">
+      <c r="J16" s="11" t="n"/>
+      <c r="K16" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L16" s="7" t="inlineStr">
@@ -2305,8 +2308,8 @@
         </is>
       </c>
       <c r="I17" s="8" t="inlineStr"/>
-      <c r="J17" s="9" t="n"/>
-      <c r="K17" s="9" t="n">
+      <c r="J17" s="11" t="n"/>
+      <c r="K17" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L17" s="7" t="inlineStr">
@@ -2404,8 +2407,8 @@
         </is>
       </c>
       <c r="I18" s="8" t="inlineStr"/>
-      <c r="J18" s="9" t="n"/>
-      <c r="K18" s="9" t="n">
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L18" s="7" t="inlineStr">
@@ -2425,7 +2428,7 @@
       </c>
       <c r="O18" s="8" t="inlineStr">
         <is>
-          <t>Canadian sheet (label signal word CAUTION). Get the US SDS from Reckitt.</t>
+          <t>Canadian sheet (CAUTION). Check the Jet-Dry we actually buy and get its US SDS from the supplier.</t>
         </is>
       </c>
       <c r="P18" s="8" t="inlineStr">
@@ -2506,10 +2509,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands</t>
         </is>
       </c>
-      <c r="J19" s="9" t="n">
+      <c r="J19" s="11" t="n">
         <v>46028</v>
       </c>
-      <c r="K19" s="9" t="n">
+      <c r="K19" s="11" t="n">
         <v>46232</v>
       </c>
       <c r="L19" s="7" t="inlineStr">
@@ -2603,10 +2606,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J20" s="9" t="n">
+      <c r="J20" s="11" t="n">
         <v>45640</v>
       </c>
-      <c r="K20" s="9" t="n">
+      <c r="K20" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L20" s="7" t="inlineStr">
@@ -2701,10 +2704,10 @@
         </is>
       </c>
       <c r="I21" s="8" t="inlineStr"/>
-      <c r="J21" s="9" t="n">
+      <c r="J21" s="11" t="n">
         <v>45982</v>
       </c>
-      <c r="K21" s="9" t="n">
+      <c r="K21" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -2766,10 +2769,10 @@
       </c>
       <c r="H22" s="8" t="inlineStr"/>
       <c r="I22" s="8" t="inlineStr"/>
-      <c r="J22" s="9" t="n">
+      <c r="J22" s="11" t="n">
         <v>42541</v>
       </c>
-      <c r="K22" s="9" t="n">
+      <c r="K22" s="11" t="n">
         <v>46315</v>
       </c>
       <c r="L22" s="7" t="inlineStr">
@@ -2870,10 +2873,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J23" s="9" t="n">
+      <c r="J23" s="11" t="n">
         <v>46067</v>
       </c>
-      <c r="K23" s="9" t="n">
+      <c r="K23" s="11" t="n">
         <v>46232</v>
       </c>
       <c r="L23" s="7" t="inlineStr">
@@ -2966,10 +2969,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands</t>
         </is>
       </c>
-      <c r="J24" s="9" t="n">
+      <c r="J24" s="11" t="n">
         <v>46255</v>
       </c>
-      <c r="K24" s="9" t="n">
+      <c r="K24" s="11" t="n">
         <v>46259</v>
       </c>
       <c r="L24" s="7" t="inlineStr">
@@ -3062,10 +3065,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J25" s="9" t="n">
+      <c r="J25" s="11" t="n">
         <v>46255</v>
       </c>
-      <c r="K25" s="9" t="n">
+      <c r="K25" s="11" t="n">
         <v>46259</v>
       </c>
       <c r="L25" s="7" t="inlineStr">
@@ -3154,10 +3157,10 @@
       <c r="G26" s="7" t="inlineStr"/>
       <c r="H26" s="8" t="inlineStr"/>
       <c r="I26" s="8" t="inlineStr"/>
-      <c r="J26" s="9" t="n">
+      <c r="J26" s="11" t="n">
         <v>46067</v>
       </c>
-      <c r="K26" s="9" t="n">
+      <c r="K26" s="11" t="n">
         <v>46232</v>
       </c>
       <c r="L26" s="7" t="inlineStr">
@@ -3258,10 +3261,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J27" s="9" t="n">
+      <c r="J27" s="11" t="n">
         <v>46255</v>
       </c>
-      <c r="K27" s="9" t="n">
+      <c r="K27" s="11" t="n">
         <v>46259</v>
       </c>
       <c r="L27" s="7" t="inlineStr">
@@ -3363,10 +3366,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands</t>
         </is>
       </c>
-      <c r="J28" s="9" t="n">
+      <c r="J28" s="11" t="n">
         <v>46107</v>
       </c>
-      <c r="K28" s="9" t="n">
+      <c r="K28" s="11" t="n">
         <v>46232</v>
       </c>
       <c r="L28" s="7" t="inlineStr">
@@ -3444,10 +3447,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands</t>
         </is>
       </c>
-      <c r="J29" s="9" t="n">
+      <c r="J29" s="11" t="n">
         <v>46107</v>
       </c>
-      <c r="K29" s="9" t="n">
+      <c r="K29" s="11" t="n">
         <v>46232</v>
       </c>
       <c r="L29" s="7" t="inlineStr">
@@ -3525,10 +3528,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J30" s="9" t="n">
+      <c r="J30" s="11" t="n">
         <v>46067</v>
       </c>
-      <c r="K30" s="9" t="n">
+      <c r="K30" s="11" t="n">
         <v>46232</v>
       </c>
       <c r="L30" s="7" t="inlineStr">
@@ -3633,10 +3636,10 @@
           <t>Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J31" s="9" t="n">
+      <c r="J31" s="11" t="n">
         <v>44989</v>
       </c>
-      <c r="K31" s="9" t="n">
+      <c r="K31" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L31" s="7" t="inlineStr">
@@ -3714,7 +3717,7 @@
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Hard Floor Santize or Sanitise (2504, 2504L, 25329, 25321 1620973, 1623626, 1631208, 1634760); 7XR2-E0GD-N00M- UVV1</t>
+          <t>Hard Floor Sanitize (2504, 2504L, 25041)</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
@@ -3730,25 +3733,26 @@
       <c r="E32" s="7" t="inlineStr"/>
       <c r="F32" s="7" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr"/>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="n"/>
       <c r="H32" s="8" t="inlineStr">
         <is>
-          <t>H412 Harmful to aquatic life with long lasting effects</t>
+          <t>H320 Causes eye irritation
+H412 Harmful to aquatic life with long lasting effects</t>
         </is>
       </c>
       <c r="I32" s="8" t="inlineStr">
         <is>
-          <t>Wash your hands</t>
-        </is>
-      </c>
-      <c r="J32" s="9" t="n">
-        <v>45062</v>
-      </c>
-      <c r="K32" s="9" t="n">
-        <v>46203</v>
+          <t>Wear eye protection; Wear protective gloves</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="n">
+        <v>45383</v>
+      </c>
+      <c r="K32" s="11" t="n">
+        <v>46317</v>
       </c>
       <c r="L32" s="7" t="inlineStr">
         <is>
@@ -3757,7 +3761,7 @@
       </c>
       <c r="M32" s="7" t="inlineStr">
         <is>
-          <t>+1(616) 453- 4451</t>
+          <t>1-866-303-6951</t>
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr">
@@ -3765,48 +3769,24 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="O32" s="8" t="inlineStr">
-        <is>
-          <t>EU-format sheet with no US OSHA classification. Get the US SDS from Bissell.</t>
-        </is>
-      </c>
+      <c r="O32" s="8" t="n"/>
       <c r="P32" s="8" t="inlineStr">
         <is>
-          <t>Inhalation: remove person to fresh air. If you are concerned, get medical advice
-Skin: wash with soap and water. If you are concerned, get medical advice
-Eyes: flush with large amounts of water. Remove contact lenses if easy to do. Continue rinsing. If signs/symptoms persist, get medical attention.
-Swallowed: rinse mouth, drink 1-2 glasses of water, do not induce vomiting. If you are concerned, get medical advice Never give anything by mouth to an unconscious person.
-Symptoms: See Section 11.1 Information on toxicological effects 4.3. Indication of any immediate medical attention and special treatment required, Not applicable</t>
-        </is>
-      </c>
-      <c r="Q32" s="8" t="inlineStr">
-        <is>
-          <t>5.1. Extinguishing media, Non-combustible. Use a fire fighting agent suitable for surrounding fire.
-Special hazards arising from the substance or mixture: None inherent in this product. During fire, gases hazardous to health may be formed.
-Advice for firefighters: In case of fire and/or explosion do not breathe fumes. Move containers from fire area if you can do so without risk.</t>
-        </is>
-      </c>
-      <c r="R32" s="8" t="inlineStr">
-        <is>
-          <t>6.1. Personal precautions, protective equipment and emergency procedures, Avoid contact with skin and eyes.
-Environmental precautions: Avoid release to the environment. Collect spillage. Dispose of contents/container in accordance with hazardous waste regulations. Do not empty into drains / surface water / ground water
-Methods and material for containment and cleaning up: Remove with liquid-absorbing material (sand, peat, sawdust). Wash away residue with plenty of water. Dispose of contaminated material as waste according to Chapter 13. 6.4. Reference to other sections, Refer to Section 8 and Section 13 for more information</t>
-        </is>
-      </c>
-      <c r="S32" s="8" t="inlineStr">
-        <is>
-          <t>7.1. Precautions for safe handling, Avoid skin and eye contact. See advice in chapter 8
-Conditions for safe storage, including any incompatibilities: Keep out of the reach of children. Store in closed original container in a well-ventilated place 7.3. Specific end use(s), See information in Section 7.1 and 7.2 for handling and storage recommendations. See Section 8 for exposure controls and personal protection recommendations.</t>
-        </is>
-      </c>
-      <c r="T32" s="8" t="inlineStr">
-        <is>
-          <t>P273 Avoid release to the environment.
-P391 Collect spillage.
-P501 Dispose of contents/container to ...</t>
-        </is>
-      </c>
-      <c r="U32" s="8" t="inlineStr"/>
+          <t>Inhalation: Move to fresh air. Get medical advice if concerned.
+Skin: Wash with soap and water. Get medical advice if concerned.
+Eyes: Flush with large amounts of water. Remove contact lenses if easy. Continue rinsing. Get medical attention if symptoms persist.
+Swallowed: Rinse mouth, drink 1-2 glasses of water. Do not induce vomiting.</t>
+        </is>
+      </c>
+      <c r="Q32" s="8" t="n"/>
+      <c r="R32" s="8" t="n"/>
+      <c r="S32" s="8" t="n"/>
+      <c r="T32" s="8" t="n"/>
+      <c r="U32" s="8" t="inlineStr">
+        <is>
+          <t>Replaced 10/22/2026: the EU-format sheet was swapped for the current US OSHA SDS (BISSELL, effective 04/01/2024).</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="45" customHeight="1">
       <c r="A33" s="7" t="n">
@@ -3836,10 +3816,10 @@
       <c r="G33" s="7" t="inlineStr"/>
       <c r="H33" s="8" t="inlineStr"/>
       <c r="I33" s="8" t="inlineStr"/>
-      <c r="J33" s="9" t="n">
+      <c r="J33" s="11" t="n">
         <v>45114</v>
       </c>
-      <c r="K33" s="9" t="n">
+      <c r="K33" s="11" t="n">
         <v>46251</v>
       </c>
       <c r="L33" s="7" t="inlineStr">
@@ -3930,8 +3910,8 @@
       </c>
       <c r="H34" s="8" t="inlineStr"/>
       <c r="I34" s="8" t="inlineStr"/>
-      <c r="J34" s="9" t="n"/>
-      <c r="K34" s="9" t="n">
+      <c r="J34" s="11" t="n"/>
+      <c r="K34" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L34" s="7" t="inlineStr">
@@ -4017,10 +3997,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J35" s="9" t="n">
+      <c r="J35" s="11" t="n">
         <v>44536</v>
       </c>
-      <c r="K35" s="9" t="n">
+      <c r="K35" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L35" s="7" t="inlineStr">
@@ -4096,10 +4076,10 @@
       <c r="G36" s="7" t="inlineStr"/>
       <c r="H36" s="8" t="inlineStr"/>
       <c r="I36" s="8" t="inlineStr"/>
-      <c r="J36" s="9" t="n">
+      <c r="J36" s="11" t="n">
         <v>45217</v>
       </c>
-      <c r="K36" s="9" t="n">
+      <c r="K36" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L36" s="7" t="inlineStr">
@@ -4200,8 +4180,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J37" s="9" t="n"/>
-      <c r="K37" s="9" t="n">
+      <c r="J37" s="11" t="n"/>
+      <c r="K37" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L37" s="7" t="inlineStr">
@@ -4307,8 +4287,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J38" s="9" t="n"/>
-      <c r="K38" s="9" t="n">
+      <c r="J38" s="11" t="n"/>
+      <c r="K38" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L38" s="7" t="inlineStr">
@@ -4415,8 +4395,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J39" s="9" t="n"/>
-      <c r="K39" s="9" t="n">
+      <c r="J39" s="11" t="n"/>
+      <c r="K39" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L39" s="7" t="inlineStr">
@@ -4532,8 +4512,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J40" s="9" t="n"/>
-      <c r="K40" s="9" t="n">
+      <c r="J40" s="11" t="n"/>
+      <c r="K40" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L40" s="7" t="inlineStr">
@@ -4624,8 +4604,8 @@
         </is>
       </c>
       <c r="I41" s="8" t="inlineStr"/>
-      <c r="J41" s="9" t="n"/>
-      <c r="K41" s="9" t="n">
+      <c r="J41" s="11" t="n"/>
+      <c r="K41" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L41" s="7" t="inlineStr">
@@ -4716,8 +4696,8 @@
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr"/>
-      <c r="J42" s="9" t="n"/>
-      <c r="K42" s="9" t="n">
+      <c r="J42" s="11" t="n"/>
+      <c r="K42" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L42" s="7" t="inlineStr">
@@ -4816,8 +4796,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J43" s="9" t="n"/>
-      <c r="K43" s="9" t="n">
+      <c r="J43" s="11" t="n"/>
+      <c r="K43" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L43" s="7" t="inlineStr">
@@ -4896,8 +4876,8 @@
       <c r="G44" s="7" t="inlineStr"/>
       <c r="H44" s="8" t="inlineStr"/>
       <c r="I44" s="8" t="inlineStr"/>
-      <c r="J44" s="9" t="n"/>
-      <c r="K44" s="9" t="n">
+      <c r="J44" s="11" t="n"/>
+      <c r="K44" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L44" s="7" t="inlineStr">
@@ -4917,7 +4897,7 @@
       </c>
       <c r="O44" s="8" t="inlineStr">
         <is>
-          <t>2011 Canadian MSDS, pre-GHS. Get the current US SDS from Reckitt.</t>
+          <t>2011 Canadian MSDS, pre-GHS. Reckitt has several "Lysol Brand III" cleaners: check the bottle we actually buy and get that exact product's US SDS.</t>
         </is>
       </c>
       <c r="P44" s="8" t="inlineStr">
@@ -5000,10 +4980,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear a mask</t>
         </is>
       </c>
-      <c r="J45" s="9" t="n">
+      <c r="J45" s="11" t="n">
         <v>45616</v>
       </c>
-      <c r="K45" s="9" t="n">
+      <c r="K45" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L45" s="7" t="inlineStr">
@@ -5104,10 +5084,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J46" s="9" t="n">
+      <c r="J46" s="11" t="n">
         <v>44813</v>
       </c>
-      <c r="K46" s="9" t="n">
+      <c r="K46" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L46" s="7" t="inlineStr">
@@ -5197,10 +5177,10 @@
       <c r="G47" s="7" t="inlineStr"/>
       <c r="H47" s="8" t="inlineStr"/>
       <c r="I47" s="8" t="inlineStr"/>
-      <c r="J47" s="9" t="n">
+      <c r="J47" s="11" t="n">
         <v>42010</v>
       </c>
-      <c r="K47" s="9" t="n">
+      <c r="K47" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L47" s="7" t="inlineStr">
@@ -5220,7 +5200,7 @@
       </c>
       <c r="O47" s="8" t="inlineStr">
         <is>
-          <t>2015 Canadian WHMIS MSDS. Get the current US SDS.</t>
+          <t>Old Canadian WHMIS MSDS. Megaloc is a Hercules (now Oatey) thread sealant: ask Oatey or the supplier for the current US SDS.</t>
         </is>
       </c>
       <c r="P47" s="8" t="inlineStr">
@@ -5286,10 +5266,10 @@
           <t>Wear eye protection; Wear safety footwear; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J48" s="9" t="n">
+      <c r="J48" s="11" t="n">
         <v>46237</v>
       </c>
-      <c r="K48" s="9" t="n">
+      <c r="K48" s="11" t="n">
         <v>46315</v>
       </c>
       <c r="L48" s="7" t="inlineStr">
@@ -5378,10 +5358,10 @@
       <c r="G49" s="7" t="inlineStr"/>
       <c r="H49" s="8" t="inlineStr"/>
       <c r="I49" s="8" t="inlineStr"/>
-      <c r="J49" s="9" t="n">
+      <c r="J49" s="11" t="n">
         <v>45765</v>
       </c>
-      <c r="K49" s="9" t="n">
+      <c r="K49" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L49" s="7" t="inlineStr">
@@ -5478,8 +5458,8 @@
           <t>Wear safety footwear; Wear protective gloves; Wear protective clothing; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J50" s="9" t="n"/>
-      <c r="K50" s="9" t="n">
+      <c r="J50" s="11" t="n"/>
+      <c r="K50" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L50" s="7" t="inlineStr">
@@ -5604,10 +5584,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J51" s="9" t="n">
+      <c r="J51" s="11" t="n">
         <v>44743</v>
       </c>
-      <c r="K51" s="9" t="n">
+      <c r="K51" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L51" s="7" t="inlineStr">
@@ -5726,8 +5706,8 @@
           <t>Wear eye protection; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J52" s="9" t="n"/>
-      <c r="K52" s="9" t="n">
+      <c r="J52" s="11" t="n"/>
+      <c r="K52" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L52" s="7" t="inlineStr">
@@ -5827,10 +5807,10 @@
         </is>
       </c>
       <c r="I53" s="8" t="inlineStr"/>
-      <c r="J53" s="9" t="n">
+      <c r="J53" s="11" t="n">
         <v>44721</v>
       </c>
-      <c r="K53" s="9" t="n">
+      <c r="K53" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L53" s="7" t="inlineStr">
@@ -5942,10 +5922,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J54" s="9" t="n">
+      <c r="J54" s="11" t="n">
         <v>45260</v>
       </c>
-      <c r="K54" s="9" t="n">
+      <c r="K54" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L54" s="7" t="inlineStr">
@@ -6043,10 +6023,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J55" s="9" t="n">
+      <c r="J55" s="11" t="n">
         <v>45749</v>
       </c>
-      <c r="K55" s="9" t="n">
+      <c r="K55" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L55" s="7" t="inlineStr">
@@ -6161,10 +6141,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands</t>
         </is>
       </c>
-      <c r="J56" s="9" t="n">
+      <c r="J56" s="11" t="n">
         <v>45293</v>
       </c>
-      <c r="K56" s="9" t="n">
+      <c r="K56" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L56" s="7" t="inlineStr">
@@ -6281,10 +6261,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J57" s="9" t="n">
+      <c r="J57" s="11" t="n">
         <v>45015</v>
       </c>
-      <c r="K57" s="9" t="n">
+      <c r="K57" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L57" s="7" t="inlineStr">
@@ -6389,8 +6369,8 @@
       <c r="G58" s="7" t="inlineStr"/>
       <c r="H58" s="8" t="inlineStr"/>
       <c r="I58" s="8" t="inlineStr"/>
-      <c r="J58" s="9" t="n"/>
-      <c r="K58" s="9" t="n">
+      <c r="J58" s="11" t="n"/>
+      <c r="K58" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L58" s="7" t="inlineStr">
@@ -6484,10 +6464,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J59" s="9" t="n">
+      <c r="J59" s="11" t="n">
         <v>45986</v>
       </c>
-      <c r="K59" s="9" t="n">
+      <c r="K59" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L59" s="7" t="inlineStr">
@@ -6578,8 +6558,8 @@
           <t>Wear eye protection; Wear protective gloves</t>
         </is>
       </c>
-      <c r="J60" s="9" t="n"/>
-      <c r="K60" s="9" t="n">
+      <c r="J60" s="11" t="n"/>
+      <c r="K60" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L60" s="7" t="inlineStr">
@@ -6679,10 +6659,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J61" s="9" t="n">
+      <c r="J61" s="11" t="n">
         <v>44813</v>
       </c>
-      <c r="K61" s="9" t="n">
+      <c r="K61" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L61" s="7" t="inlineStr">
@@ -6776,8 +6756,8 @@
           <t>Wear eye protection; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J62" s="9" t="n"/>
-      <c r="K62" s="9" t="n">
+      <c r="J62" s="11" t="n"/>
+      <c r="K62" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L62" s="7" t="inlineStr">
@@ -6860,8 +6840,8 @@
       <c r="G63" s="7" t="inlineStr"/>
       <c r="H63" s="8" t="inlineStr"/>
       <c r="I63" s="8" t="inlineStr"/>
-      <c r="J63" s="9" t="n"/>
-      <c r="K63" s="9" t="n">
+      <c r="J63" s="11" t="n"/>
+      <c r="K63" s="11" t="n">
         <v>46231</v>
       </c>
       <c r="L63" s="7" t="inlineStr">
@@ -6944,10 +6924,10 @@
       </c>
       <c r="H64" s="8" t="inlineStr"/>
       <c r="I64" s="8" t="inlineStr"/>
-      <c r="J64" s="9" t="n">
+      <c r="J64" s="11" t="n">
         <v>45153</v>
       </c>
-      <c r="K64" s="9" t="n">
+      <c r="K64" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L64" s="7" t="inlineStr">
@@ -7044,10 +7024,10 @@
           <t>Wash your hands</t>
         </is>
       </c>
-      <c r="J65" s="9" t="n">
+      <c r="J65" s="11" t="n">
         <v>46100</v>
       </c>
-      <c r="K65" s="9" t="n">
+      <c r="K65" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L65" s="7" t="inlineStr">
@@ -7139,10 +7119,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands; Wear respiratory protection; Use barrier cream</t>
         </is>
       </c>
-      <c r="J66" s="9" t="n">
+      <c r="J66" s="11" t="n">
         <v>45943</v>
       </c>
-      <c r="K66" s="9" t="n">
+      <c r="K66" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L66" s="7" t="inlineStr">
@@ -7260,10 +7240,10 @@
           <t>Wear eye protection; Wear protective clothing</t>
         </is>
       </c>
-      <c r="J67" s="9" t="n">
+      <c r="J67" s="11" t="n">
         <v>44862</v>
       </c>
-      <c r="K67" s="9" t="n">
+      <c r="K67" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L67" s="7" t="inlineStr">
@@ -7399,10 +7379,10 @@
         </is>
       </c>
       <c r="I68" s="8" t="inlineStr"/>
-      <c r="J68" s="9" t="n">
+      <c r="J68" s="11" t="n">
         <v>41604</v>
       </c>
-      <c r="K68" s="9" t="n">
+      <c r="K68" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L68" s="7" t="inlineStr">
@@ -7508,8 +7488,8 @@
       <c r="G69" s="7" t="inlineStr"/>
       <c r="H69" s="8" t="inlineStr"/>
       <c r="I69" s="8" t="inlineStr"/>
-      <c r="J69" s="9" t="n"/>
-      <c r="K69" s="9" t="n">
+      <c r="J69" s="11" t="n"/>
+      <c r="K69" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L69" s="7" t="inlineStr">
@@ -7524,14 +7504,10 @@
       </c>
       <c r="N69" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O69" s="8" t="inlineStr">
-        <is>
-          <t>Duplicate of ID 3370841 (Simple Green All-Purpose). Keep one.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O69" s="8" t="n"/>
       <c r="P69" s="8" t="inlineStr">
         <is>
           <t>General: No expected hazards
@@ -7577,7 +7553,11 @@
         </is>
       </c>
       <c r="T69" s="8" t="inlineStr"/>
-      <c r="U69" s="8" t="inlineStr"/>
+      <c r="U69" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Duplicate of ID 3370841 (Simple Green All-Purpose).</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="45" customHeight="1">
       <c r="A70" s="7" t="n">
@@ -7611,8 +7591,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands</t>
         </is>
       </c>
-      <c r="J70" s="9" t="n"/>
-      <c r="K70" s="9" t="n">
+      <c r="J70" s="11" t="n"/>
+      <c r="K70" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L70" s="7" t="inlineStr">
@@ -7691,8 +7671,8 @@
       <c r="G71" s="7" t="inlineStr"/>
       <c r="H71" s="8" t="inlineStr"/>
       <c r="I71" s="8" t="inlineStr"/>
-      <c r="J71" s="9" t="n"/>
-      <c r="K71" s="9" t="n">
+      <c r="J71" s="11" t="n"/>
+      <c r="K71" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L71" s="7" t="inlineStr">
@@ -7789,10 +7769,10 @@
         </is>
       </c>
       <c r="I72" s="8" t="inlineStr"/>
-      <c r="J72" s="9" t="n">
+      <c r="J72" s="11" t="n">
         <v>45890</v>
       </c>
-      <c r="K72" s="9" t="n">
+      <c r="K72" s="11" t="n">
         <v>46315</v>
       </c>
       <c r="L72" s="7" t="inlineStr">
@@ -7903,10 +7883,10 @@
       </c>
       <c r="H73" s="8" t="inlineStr"/>
       <c r="I73" s="8" t="inlineStr"/>
-      <c r="J73" s="9" t="n">
+      <c r="J73" s="11" t="n">
         <v>45012</v>
       </c>
-      <c r="K73" s="9" t="n">
+      <c r="K73" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L73" s="7" t="inlineStr">
@@ -8003,10 +7983,10 @@
         </is>
       </c>
       <c r="I74" s="8" t="inlineStr"/>
-      <c r="J74" s="9" t="n">
+      <c r="J74" s="11" t="n">
         <v>44593</v>
       </c>
-      <c r="K74" s="9" t="n">
+      <c r="K74" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L74" s="7" t="inlineStr">
@@ -8115,10 +8095,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J75" s="9" t="n">
+      <c r="J75" s="11" t="n">
         <v>45088</v>
       </c>
-      <c r="K75" s="9" t="n">
+      <c r="K75" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L75" s="7" t="inlineStr">
@@ -8133,14 +8113,10 @@
       </c>
       <c r="N75" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O75" s="8" t="inlineStr">
-        <is>
-          <t>Older revision (2023) of Slide Mold Cleaner 4. ID 3091972 is the 2025 revision.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O75" s="8" t="n"/>
       <c r="P75" s="8" t="inlineStr">
         <is>
           <t>General: In all cases of doubt, or when symptoms persist, seek medical attention. Never give anything by mouth to an unconscious person.
@@ -8200,7 +8176,11 @@
 P501 Dispose of contents/container to ...</t>
         </is>
       </c>
-      <c r="U75" s="8" t="inlineStr"/>
+      <c r="U75" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Older 2023 revision; current is ID 3091972 (2025).</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="45" customHeight="1">
       <c r="A76" s="7" t="n">
@@ -8246,10 +8226,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J76" s="9" t="n">
+      <c r="J76" s="11" t="n">
         <v>45679</v>
       </c>
-      <c r="K76" s="9" t="n">
+      <c r="K76" s="11" t="n">
         <v>46266</v>
       </c>
       <c r="L76" s="7" t="inlineStr">
@@ -8366,10 +8346,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J77" s="9" t="n">
+      <c r="J77" s="11" t="n">
         <v>45406</v>
       </c>
-      <c r="K77" s="9" t="n">
+      <c r="K77" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L77" s="7" t="inlineStr">
@@ -8488,10 +8468,10 @@
         </is>
       </c>
       <c r="I78" s="8" t="inlineStr"/>
-      <c r="J78" s="9" t="n">
+      <c r="J78" s="11" t="n">
         <v>45868</v>
       </c>
-      <c r="K78" s="9" t="n">
+      <c r="K78" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L78" s="7" t="inlineStr">
@@ -8607,10 +8587,10 @@
         </is>
       </c>
       <c r="I79" s="8" t="inlineStr"/>
-      <c r="J79" s="9" t="n">
+      <c r="J79" s="11" t="n">
         <v>42005</v>
       </c>
-      <c r="K79" s="9" t="n">
+      <c r="K79" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L79" s="7" t="inlineStr">
@@ -8625,14 +8605,10 @@
       </c>
       <c r="N79" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O79" s="8" t="inlineStr">
-        <is>
-          <t>Older revision (2015) of Slide Quick Lecithin. ID 2967305 is the 2025 revision.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O79" s="8" t="n"/>
       <c r="P79" s="8" t="inlineStr">
         <is>
           <t>Eyes: Rinse thoroughly with plenty of water, also under the eyelids. If eye irritation persists: Get medical advice/attention.
@@ -8684,7 +8660,11 @@
 P410+P412 Protect from sunlight.  Do not expose to temperatures exceeding 50 °C/122 °F.</t>
         </is>
       </c>
-      <c r="U79" s="8" t="inlineStr"/>
+      <c r="U79" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Older 2015 revision; current is ID 2967305 (2025).</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="45" customHeight="1">
       <c r="A80" s="7" t="n">
@@ -8728,10 +8708,10 @@
         </is>
       </c>
       <c r="I80" s="8" t="inlineStr"/>
-      <c r="J80" s="9" t="n">
+      <c r="J80" s="11" t="n">
         <v>45328</v>
       </c>
-      <c r="K80" s="9" t="n">
+      <c r="K80" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L80" s="7" t="inlineStr">
@@ -8854,10 +8834,10 @@
         </is>
       </c>
       <c r="I81" s="8" t="inlineStr"/>
-      <c r="J81" s="9" t="n">
+      <c r="J81" s="11" t="n">
         <v>45950</v>
       </c>
-      <c r="K81" s="9" t="n">
+      <c r="K81" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L81" s="7" t="inlineStr">
@@ -8977,10 +8957,10 @@
         </is>
       </c>
       <c r="I82" s="8" t="inlineStr"/>
-      <c r="J82" s="9" t="n">
+      <c r="J82" s="11" t="n">
         <v>45721</v>
       </c>
-      <c r="K82" s="9" t="n">
+      <c r="K82" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L82" s="7" t="inlineStr">
@@ -9088,10 +9068,10 @@
         </is>
       </c>
       <c r="I83" s="8" t="inlineStr"/>
-      <c r="J83" s="9" t="n">
+      <c r="J83" s="11" t="n">
         <v>45721</v>
       </c>
-      <c r="K83" s="9" t="n">
+      <c r="K83" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L83" s="7" t="inlineStr">
@@ -9106,14 +9086,10 @@
       </c>
       <c r="N83" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O83" s="8" t="inlineStr">
-        <is>
-          <t>Duplicate of ID 3370926 (White Rhino). Keep one.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O83" s="8" t="n"/>
       <c r="P83" s="8" t="inlineStr">
         <is>
           <t>General: In all cases of doubt, or when symptoms persist, seek medical attention. Never give anything by mouth to an unconscious person.
@@ -9167,7 +9143,11 @@
 P501 Dispose of contents/container to ...</t>
         </is>
       </c>
-      <c r="U83" s="8" t="inlineStr"/>
+      <c r="U83" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Duplicate of ID 3370926 (White Rhino).</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="45" customHeight="1">
       <c r="A84" s="7" t="n">
@@ -9201,10 +9181,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J84" s="9" t="n">
+      <c r="J84" s="11" t="n">
         <v>39162</v>
       </c>
-      <c r="K84" s="9" t="n">
+      <c r="K84" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L84" s="7" t="inlineStr">
@@ -9219,14 +9199,10 @@
       </c>
       <c r="N84" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O84" s="8" t="inlineStr">
-        <is>
-          <t>Pre-GHS MSDS from 2007. The 2018 GHS sheet for the same paint is ID 3370806, so archive this one.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O84" s="8" t="n"/>
       <c r="P84" s="8" t="inlineStr">
         <is>
           <t>Eyes: Immediately flush eyes with water for at least 15 minutes. If irritation develops get medical attention.
@@ -9256,7 +9232,11 @@
         </is>
       </c>
       <c r="T84" s="8" t="inlineStr"/>
-      <c r="U84" s="8" t="inlineStr"/>
+      <c r="U84" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Superseded by ID 3370806 (2018 GHS SDS for the same paint).</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="45" customHeight="1">
       <c r="A85" s="7" t="n">
@@ -9307,10 +9287,10 @@
           <t>Wear eye protection; Wear protective gloves; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J85" s="9" t="n">
+      <c r="J85" s="11" t="n">
         <v>43199</v>
       </c>
-      <c r="K85" s="9" t="n">
+      <c r="K85" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L85" s="7" t="inlineStr">
@@ -9429,8 +9409,8 @@
         </is>
       </c>
       <c r="I86" s="8" t="inlineStr"/>
-      <c r="J86" s="9" t="n"/>
-      <c r="K86" s="9" t="n">
+      <c r="J86" s="11" t="n"/>
+      <c r="K86" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L86" s="7" t="inlineStr">
@@ -9445,14 +9425,10 @@
       </c>
       <c r="N86" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O86" s="8" t="inlineStr">
-        <is>
-          <t>Spanish-language copy. The English version is ID 3007032, so archive this one.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O86" s="8" t="n"/>
       <c r="P86" s="8" t="inlineStr">
         <is>
           <t>Swallowed: Llamar inmediatamente al médico o Centro de Toxicología. Enjuagarse la boca. No administrar nunca líquidos a una persona inconsciente. En caso de vómito, mantener la cabeza a un nivel más bajo que el estómago para evitar que el vómito entre en los pulmones.
@@ -9509,7 +9485,11 @@
 P410+P412 Protect from sunlight.  Do not expose to temperatures exceeding 50 °C/122 °F.</t>
         </is>
       </c>
-      <c r="U86" s="8" t="inlineStr"/>
+      <c r="U86" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Spanish-language copy; the English SDS is ID 3007032.</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="45" customHeight="1">
       <c r="A87" s="7" t="n">
@@ -9551,8 +9531,8 @@
         </is>
       </c>
       <c r="I87" s="8" t="inlineStr"/>
-      <c r="J87" s="9" t="n"/>
-      <c r="K87" s="9" t="n">
+      <c r="J87" s="11" t="n"/>
+      <c r="K87" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L87" s="7" t="inlineStr">
@@ -9658,10 +9638,10 @@
       </c>
       <c r="H88" s="8" t="inlineStr"/>
       <c r="I88" s="8" t="inlineStr"/>
-      <c r="J88" s="9" t="n">
+      <c r="J88" s="11" t="n">
         <v>45995</v>
       </c>
-      <c r="K88" s="9" t="n">
+      <c r="K88" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L88" s="7" t="inlineStr">
@@ -9752,10 +9732,10 @@
       </c>
       <c r="H89" s="8" t="inlineStr"/>
       <c r="I89" s="8" t="inlineStr"/>
-      <c r="J89" s="9" t="n">
+      <c r="J89" s="11" t="n">
         <v>42122</v>
       </c>
-      <c r="K89" s="9" t="n">
+      <c r="K89" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L89" s="7" t="inlineStr">
@@ -9773,11 +9753,7 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="O89" s="8" t="inlineStr">
-        <is>
-          <t>Same PDF as ID 3091976. Archive one of the two.</t>
-        </is>
-      </c>
+      <c r="O89" s="8" t="n"/>
       <c r="P89" s="8" t="inlineStr">
         <is>
           <t>First aid measures for different exposure routes
@@ -9862,10 +9838,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J90" s="9" t="n">
+      <c r="J90" s="11" t="n">
         <v>42122</v>
       </c>
-      <c r="K90" s="9" t="n">
+      <c r="K90" s="11" t="n">
         <v>46266</v>
       </c>
       <c r="L90" s="7" t="inlineStr">
@@ -9880,14 +9856,10 @@
       </c>
       <c r="N90" s="7" t="inlineStr">
         <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="O90" s="8" t="inlineStr">
-        <is>
-          <t>Same PDF as ID 2967291. Archive one of the two.</t>
-        </is>
-      </c>
+          <t>Archived</t>
+        </is>
+      </c>
+      <c r="O90" s="8" t="n"/>
       <c r="P90" s="8" t="inlineStr">
         <is>
           <t>First aid measures for different exposure routes
@@ -9948,7 +9920,11 @@
 P405 Store locked up.</t>
         </is>
       </c>
-      <c r="U90" s="8" t="inlineStr"/>
+      <c r="U90" s="8" t="inlineStr">
+        <is>
+          <t>Archived 10/22/2026: Same PDF as ID 2967291 (TUFF KOTE).</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="45" customHeight="1">
       <c r="A91" s="7" t="n">
@@ -9982,10 +9958,10 @@
       </c>
       <c r="H91" s="8" t="inlineStr"/>
       <c r="I91" s="8" t="inlineStr"/>
-      <c r="J91" s="9" t="n">
+      <c r="J91" s="11" t="n">
         <v>43831</v>
       </c>
-      <c r="K91" s="9" t="n">
+      <c r="K91" s="11" t="n">
         <v>46317</v>
       </c>
       <c r="L91" s="7" t="inlineStr">
@@ -10071,8 +10047,8 @@
           <t>Wear eye protection; Wear protective gloves; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J92" s="9" t="n"/>
-      <c r="K92" s="9" t="n">
+      <c r="J92" s="11" t="n"/>
+      <c r="K92" s="11" t="n">
         <v>46316</v>
       </c>
       <c r="L92" s="7" t="inlineStr">
@@ -10145,8 +10121,8 @@
       <c r="G93" s="7" t="inlineStr"/>
       <c r="H93" s="8" t="inlineStr"/>
       <c r="I93" s="8" t="inlineStr"/>
-      <c r="J93" s="9" t="n"/>
-      <c r="K93" s="9" t="n">
+      <c r="J93" s="11" t="n"/>
+      <c r="K93" s="11" t="n">
         <v>46316</v>
       </c>
       <c r="L93" s="7" t="inlineStr">
@@ -10219,10 +10195,10 @@
       <c r="G94" s="7" t="inlineStr"/>
       <c r="H94" s="8" t="inlineStr"/>
       <c r="I94" s="8" t="inlineStr"/>
-      <c r="J94" s="9" t="n">
+      <c r="J94" s="11" t="n">
         <v>42221</v>
       </c>
-      <c r="K94" s="9" t="n">
+      <c r="K94" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L94" s="7" t="inlineStr">
@@ -10320,10 +10296,10 @@
           <t>Wear eye protection; Wear safety footwear; Wear protective gloves; Wear protective clothing; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J95" s="9" t="n">
+      <c r="J95" s="11" t="n">
         <v>45995</v>
       </c>
-      <c r="K95" s="9" t="n">
+      <c r="K95" s="11" t="n">
         <v>46224</v>
       </c>
       <c r="L95" s="7" t="inlineStr">
@@ -10425,10 +10401,10 @@
           <t>Wash your hands</t>
         </is>
       </c>
-      <c r="J96" s="9" t="n">
+      <c r="J96" s="11" t="n">
         <v>46002</v>
       </c>
-      <c r="K96" s="9" t="n">
+      <c r="K96" s="11" t="n">
         <v>46251</v>
       </c>
       <c r="L96" s="7" t="inlineStr">
@@ -10519,10 +10495,10 @@
         </is>
       </c>
       <c r="I97" s="8" t="inlineStr"/>
-      <c r="J97" s="9" t="n">
+      <c r="J97" s="11" t="n">
         <v>44120</v>
       </c>
-      <c r="K97" s="9" t="n">
+      <c r="K97" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L97" s="7" t="inlineStr">
@@ -10624,10 +10600,10 @@
           <t>Wear eye protection; Wear protective gloves; Wash your hands; Wear respiratory protection</t>
         </is>
       </c>
-      <c r="J98" s="9" t="n">
+      <c r="J98" s="11" t="n">
         <v>43621</v>
       </c>
-      <c r="K98" s="9" t="n">
+      <c r="K98" s="11" t="n">
         <v>46203</v>
       </c>
       <c r="L98" s="7" t="inlineStr">
@@ -10714,10 +10690,10 @@
       <c r="G99" s="7" t="inlineStr"/>
       <c r="H99" s="8" t="inlineStr"/>
       <c r="I99" s="8" t="inlineStr"/>
-      <c r="J99" s="9" t="n">
+      <c r="J99" s="11" t="n">
         <v>42060</v>
       </c>
-      <c r="K99" s="9" t="n">
+      <c r="K99" s="11" t="n">
         <v>46289</v>
       </c>
       <c r="L99" s="7" t="inlineStr">
@@ -10764,8 +10740,115 @@
       <c r="T99" s="8" t="inlineStr"/>
       <c r="U99" s="8" t="inlineStr"/>
     </row>
+    <row r="100" ht="45" customHeight="1">
+      <c r="A100" s="7" t="n">
+        <v>4000001</v>
+      </c>
+      <c r="B100" s="8" t="inlineStr">
+        <is>
+          <t>Slide Resin Remover Aerosol (41914)</t>
+        </is>
+      </c>
+      <c r="C100" s="8" t="inlineStr">
+        <is>
+          <t>Slide Products Inc</t>
+        </is>
+      </c>
+      <c r="D100" s="7" t="inlineStr">
+        <is>
+          <t>Mold release &amp; mold care</t>
+        </is>
+      </c>
+      <c r="E100" s="7" t="inlineStr">
+        <is>
+          <t>Press floor, mold cleaning</t>
+        </is>
+      </c>
+      <c r="F100" s="7" t="inlineStr">
+        <is>
+          <t>Danger</t>
+        </is>
+      </c>
+      <c r="G100" s="7" t="inlineStr">
+        <is>
+          <t>GHS02, GHS07, GHS08</t>
+        </is>
+      </c>
+      <c r="H100" s="8" t="inlineStr">
+        <is>
+          <t>H223 Flammable aerosol
+H332 Harmful if inhaled
+H315 Causes skin irritation
+H319 Causes serious eye irritation
+H360 May damage fertility or the unborn child
+H335 May cause respiratory irritation
+H336 May cause drowsiness or dizziness
+H373 May cause damage to organs through prolonged or repeated exposure</t>
+        </is>
+      </c>
+      <c r="I100" s="8" t="inlineStr">
+        <is>
+          <t>Wear eye protection; Wear protective gloves</t>
+        </is>
+      </c>
+      <c r="J100" s="11" t="n">
+        <v>42005</v>
+      </c>
+      <c r="K100" s="11" t="n">
+        <v>46317</v>
+      </c>
+      <c r="L100" s="7" t="inlineStr">
+        <is>
+          <t>4000001.pdf</t>
+        </is>
+      </c>
+      <c r="M100" s="7" t="inlineStr">
+        <is>
+          <t>1-800-535-5053</t>
+        </is>
+      </c>
+      <c r="N100" s="7" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="O100" s="8" t="n"/>
+      <c r="P100" s="8" t="inlineStr">
+        <is>
+          <t>General: If exposed or concerned, get medical advice.
+Eyes: Flush with plenty of water for at least 15 minutes, removing contact lenses after the first flush. Call a physician immediately.
+Skin: Wash with soap and water. Remove contaminated clothing and shoes. Get medical advice if irritation occurs.
+Inhalation: Move to fresh air and keep at rest.
+Swallowed: Rinse mouth, then drink plenty of water.</t>
+        </is>
+      </c>
+      <c r="Q100" s="8" t="inlineStr">
+        <is>
+          <t>Extinguishing media: Dry chemical, foam, carbon dioxide. Do not use water.
+Special hazards: Aerosol cans may rupture violently above 120°F. Burning forms HCl and traces of phosgene.
+Firefighters: Self-contained breathing apparatus and full protective gear.</t>
+        </is>
+      </c>
+      <c r="R100" s="8" t="inlineStr">
+        <is>
+          <t>Remove all ignition sources. Move a leaking can outside to a disposal area. Collect in closed containers for disposal.</t>
+        </is>
+      </c>
+      <c r="S100" s="8" t="inlineStr">
+        <is>
+          <t>Read the SDS before first use. Use only with good ventilation; do not breathe vapors or spray. Keep away from heat, sparks and flames; no smoking. Do not spray on painted surfaces or floors.
+Storage: Store locked up in a cool, dry, well-ventilated place, out of sunlight, below 120°F.</t>
+        </is>
+      </c>
+      <c r="T100" s="8" t="n"/>
+      <c r="U100" s="8" t="inlineStr">
+        <is>
+          <t>Added 10/22/2026 (named in MIOSHA Item 9). Contains n-propyl bromide and NMP, which are reproductive toxicants. Neoprene gloves per Section 8. If the bulk can (419BULK) is also used, add its SDS too.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:U99"/>
+  <autoFilter ref="A1:U100"/>
   <dataValidations count="3">
     <dataValidation sqref="D2:D2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>Lists!$A$2:$A$7</formula1>

</xml_diff>

<commit_message>
SDS register: fill in missing revision dates for Loctite 515 (x2) and Simple Green APC
The PDFs already in the library are the current US revisions
(Henkel rev 012.0, 06/04/2025; Sunshine Makers 13000-25A, 10/01/2025);
the register just had the dates blank.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013w8SjJa87snYar4uybgyE4
</commit_message>
<xml_diff>
--- a/sds/SDS-Register.xlsx
+++ b/sds/SDS-Register.xlsx
@@ -4512,7 +4512,9 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands; Wear a face shield; Wear respiratory protection; Use protective apron</t>
         </is>
       </c>
-      <c r="J40" s="11" t="n"/>
+      <c r="J40" s="11" t="n">
+        <v>45812</v>
+      </c>
       <c r="K40" s="11" t="n">
         <v>46289</v>
       </c>
@@ -4696,7 +4698,9 @@
         </is>
       </c>
       <c r="I42" s="8" t="inlineStr"/>
-      <c r="J42" s="11" t="n"/>
+      <c r="J42" s="11" t="n">
+        <v>45812</v>
+      </c>
       <c r="K42" s="11" t="n">
         <v>46289</v>
       </c>
@@ -7591,7 +7595,9 @@
           <t>Wear eye protection; Wear protective gloves; Wear protective clothing; Wash your hands</t>
         </is>
       </c>
-      <c r="J70" s="11" t="n"/>
+      <c r="J70" s="11" t="n">
+        <v>45931</v>
+      </c>
       <c r="K70" s="11" t="n">
         <v>46317</v>
       </c>

</xml_diff>

<commit_message>
SDS library: replace Prominence Heavy Duty Floor Cleaner with current US SDS
2018 Canadian (WHMIS) sheet swapped for Diversey US SDS MS0802259,
v01.0, 2025-12-04. Register row updated: revision date, hazard and
precautionary statements, first aid, emergency phone; Date Added set
so it shows on the New & revised notice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013w8SjJa87snYar4uybgyE4
</commit_message>
<xml_diff>
--- a/sds/SDS-Register.xlsx
+++ b/sds/SDS-Register.xlsx
@@ -6556,15 +6556,22 @@
           <t>GHS07</t>
         </is>
       </c>
-      <c r="H60" s="8" t="inlineStr"/>
+      <c r="H60" s="8" t="inlineStr">
+        <is>
+          <t>H315 Causes skin irritation
+H319 Causes serious eye irritation</t>
+        </is>
+      </c>
       <c r="I60" s="8" t="inlineStr">
         <is>
           <t>Wear eye protection; Wear protective gloves</t>
         </is>
       </c>
-      <c r="J60" s="11" t="n"/>
+      <c r="J60" s="11" t="n">
+        <v>45995</v>
+      </c>
       <c r="K60" s="11" t="n">
-        <v>46224</v>
+        <v>46321</v>
       </c>
       <c r="L60" s="7" t="inlineStr">
         <is>
@@ -6573,7 +6580,7 @@
       </c>
       <c r="M60" s="7" t="inlineStr">
         <is>
-          <t>1-800-668-7171</t>
+          <t>1-800-851-7145</t>
         </is>
       </c>
       <c r="N60" s="7" t="inlineStr">
@@ -6584,43 +6591,47 @@
       <c r="O60" s="8" t="inlineStr"/>
       <c r="P60" s="8" t="inlineStr">
         <is>
-          <t>Eyes: Rinse cautiously with water for several minutes. Remove contact lenses, if present and easy to do. Continue rinsing for at least 15 minutes. If eye irritation persists: Get medical advice/attention. Rinse with plenty of water If irritation occurs and persists, get medical attention
-Skin: Wash with plenty of soap and water. No specific first aid measures are required Inhalation: No specific first aid measures are required
-Skin: Get medical advice/attention Inhalation: No specific first aid measures are required.
-Swallowed: Rinse mouth. Drink a cupful of milk or water
-Symptoms: No information available
-Medical attention: Not applicable Aggravated Medical Conditions: None known. Diluted Product
-Swallowed: Rinse mouth with water</t>
+          <t>Undiluted product:
+Eyes: Rinse cautiously with water for several minutes. Remove contact lenses, if present and easy to do. Continue rinsing for at least 15 minutes. If eye irritation persists: Get medical advice/attention.
+Skin: Wash with plenty of soap and water for at least 15 minutes. If skin irritation occurs: Get medical advice/attention.
+Inhalation: No specific first aid measures are required.
+Swallowed: Call a Poison Center (1-800-851-7145) or doctor if you feel unwell.
+Diluted product: Eyes: rinse with plenty of water. Skin and inhalation: no specific measures required.</t>
         </is>
       </c>
       <c r="Q60" s="8" t="inlineStr">
         <is>
           <t>Specific methods: No special methods required
 Suitable extinguishing agents: The product is not flammable. Extinguish fire using agent suitable for surrounding fire.
-Special Hazards caused by the Material: Not applicable.
-Advice for firefighters: As in any fire, wear self-contained breathing apparatus pressure-demand, MSHA/NIOSH (approved or equivalent) and full protective gear.
-Unsuitable extinguishing: No information available</t>
+Specific hazards: None known.
+Advice for firefighters: As in any fire, wear self-contained breathing apparatus pressure-demand, MSHA/NIOSH (approved or equivalent) and full protective gear.</t>
         </is>
       </c>
       <c r="R60" s="8" t="inlineStr">
         <is>
-          <t>Personal precautions, protective equipment and emergency procedures: Put on appropriate personal protective equipment (see Section 8.).
-Methods and material for containment and cleaning up: - large spillage. Absorb spill with inert material (e.g. dry sand or earth), then place in and clean-up methods a chemical waste container. Use a water rinse for final clean-up.</t>
+          <t>Personal precautions: Put on appropriate personal protective equipment (see Section 8).
+Containment and clean-up: Absorb large spills with inert material (e.g. dry sand or earth), then place in a chemical waste container. Use a water rinse for final clean-up.</t>
         </is>
       </c>
       <c r="S60" s="8" t="inlineStr">
         <is>
-          <t>Precautions for safe handling: Avoid contact with skin, eyes and clothing. Do not taste or swallow. Remove and wash contaminated clothing and footwear before re-use. Wash thoroughly after handling. Product residue may remain on/in empty containers. All precautions for handling the product must be used in handling the empty container and residue. FOR COMMERCIAL AND INDUSTRIAL USE ONLY.
-Conditions for safe storage, including any incompatibilities: Protect from freezing. Keep tightly closed in a dry, cool and well-ventilated place. KEEP OUT OF REACH OF CHILDREN Aerosol Level (if applicable) Not applicable.</t>
+          <t>Handling: Avoid contact with eyes. FOR COMMERCIAL AND INDUSTRIAL USE ONLY.
+Storage: Keep tightly closed in a dry, cool and well-ventilated place.</t>
         </is>
       </c>
       <c r="T60" s="8" t="inlineStr">
         <is>
-          <t>P337+P313 If eye irritation persists:  Get medical advice/attention.
-P363 Wash contaminated clothing before reuse.</t>
-        </is>
-      </c>
-      <c r="U60" s="8" t="inlineStr"/>
+          <t>Avoid contact with eyes, skin and clothing. Wash affected areas thoroughly after handling. Wear chemical-splash goggles and chemical-resistant gloves.
+IF IN EYES: Rinse cautiously with water for at least 15 minutes. If eye irritation persists: Get medical advice/attention.
+IF ON SKIN: Wash with plenty of soap and water. If skin irritation occurs: Get medical advice/attention.
+Take off contaminated clothing and wash it before reuse.</t>
+        </is>
+      </c>
+      <c r="U60" s="8" t="inlineStr">
+        <is>
+          <t>Replaced 10/26/2026: 2018 Canadian (WHMIS) sheet swapped for the current US SDS (Diversey MS0802259, v01.0, 2025-12-04). Diluted 1:256 it is not classified as hazardous; PPE above is for the concentrate.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="45" customHeight="1">
       <c r="A61" s="7" t="n">

</xml_diff>

<commit_message>
SDS register: fix Tuff Kote pictograms, add hazard statements and review flag
Pictograms were GHS05 (corrosion); the SDS and the pail label both show
GHS07 (exclamation mark). Flagged for a current SDS covering the 5-gal
TK-150-5 pail.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013w8SjJa87snYar4uybgyE4
</commit_message>
<xml_diff>
--- a/sds/SDS-Register.xlsx
+++ b/sds/SDS-Register.xlsx
@@ -9744,10 +9744,19 @@
       </c>
       <c r="G89" s="7" t="inlineStr">
         <is>
-          <t>GHS02, GHS05, GHS08</t>
-        </is>
-      </c>
-      <c r="H89" s="8" t="inlineStr"/>
+          <t>GHS02, GHS07, GHS08</t>
+        </is>
+      </c>
+      <c r="H89" s="8" t="inlineStr">
+        <is>
+          <t>H224 Extremely flammable liquid and vapour
+H304 May be fatal if swallowed and enters airways
+H315 Causes skin irritation
+H319 Causes serious eye irritation
+H335 May cause respiratory irritation
+H336 May cause drowsiness or dizziness</t>
+        </is>
+      </c>
       <c r="I89" s="8" t="inlineStr"/>
       <c r="J89" s="11" t="n">
         <v>42122</v>
@@ -9770,7 +9779,11 @@
           <t>Active</t>
         </is>
       </c>
-      <c r="O89" s="8" t="n"/>
+      <c r="O89" s="8" t="inlineStr">
+        <is>
+          <t>On site as 5-gal pail TK-150-5 (date code 9/19/22). The 2015 SDS on file is for the aerosol at Nanoplas's old address; the pail label shows Highly flammable (Cat 2), UN1993 PG II and the Grandville address. Request the current US SDS for TK-150 from Nanoplas (616-452-3707, nanomoldcoating.com/sds-request).</t>
+        </is>
+      </c>
       <c r="P89" s="8" t="inlineStr">
         <is>
           <t>First aid measures for different exposure routes

</xml_diff>